<commit_message>
Enhance BufferComposition with comprehensive pH specification
- Replace single 'ph' field with 'buffer_ph' (pH before sample addition)
- Add 'final_sample_ph' (pH after all components added)
- Add pH measurement context fields:
  - ph_measurement_temperature (°C)
  - ph_measurement_method (electrode type, calibration)
  - ph_stability_notes (stability during experiment)
  - ionic_strength (mM at measurement)

This addresses issue #19 by distinguishing between buffer pH and final
sample pH, which can differ by 0.3-0.8 pH units due to protein
contributions, metal ion binding, and cofactor effects.

Updated all 17 test examples to use new buffer_ph field.
Regenerated all schema artifacts and validated examples.

🤖 Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Chris Mungall <cmungall@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/excel/biostride.xlsx
+++ b/assets/excel/biostride.xlsx
@@ -1499,26 +1499,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ph</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>buffer_ph</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>final_sample_ph</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ph_measurement_temperature</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ph_measurement_method</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ph_stability_notes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ionic_strength</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>components</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>additives</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Fix all validation issues in functional annotation examples
- Add missing enum values (zinc_binding, disordered, intact, cosmic, clinvar)
- Fix all CURIE prefixes to use 'biostride:' namespace
- Add missing IDs to all annotation objects
- Fix invalid enum values in examples
- Update inlined directives for complex objects

Main examples now validate successfully:
- Sample-with-functional-annotations.yaml ✅
- AggregatedProteinView-example.yaml ✅
- Dataset-loosenin-bioenergy.yaml ✅

🤖 Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/biostride.xlsx
+++ b/assets/excel/biostride.xlsx
@@ -2593,13 +2593,13 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
+      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed"</formula1>
+      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>

</xml_diff>